<commit_message>
hotels and recreation 검수
</commit_message>
<xml_diff>
--- a/Data/Hotels and Recreation - 3814336747/Hotels and Recreation - 3814336747.xlsx
+++ b/Data/Hotels and Recreation - 3814336747/Hotels and Recreation - 3814336747.xlsx
@@ -15657,8 +15657,10 @@
       <c r="E5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>23</v>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">행사가 잘못 풀림</t>
+        </is>
       </c>
     </row>
     <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15742,8 +15744,10 @@
       <c r="E10" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>46</v>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">동전 밀어내기 기계</t>
+        </is>
       </c>
     </row>
     <row r="11" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15810,8 +15814,10 @@
       <c r="E14" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>60</v>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">카지노를 상대로 21에 도전해 보세요. 카지노 게임 중에서도 운영자에게 돌아가는 이익이 가장 적은 편이라, 진지하게 도박을 즐기는 손님들이 찾습니다.\n\n의자가 필요합니다. 플레이어는 앉아서 게임을 하므로, 테이블 바로 옆에 플레이어마다 의자나 걸상을 하나씩 놓으세요. 최대 4명까지 이용할 수 있으며, 딜러는 필요 없습니다. 호텔 투숙객은 설정된 판돈을 자신의 예산에서 지불하고, 정착민은 재미로 즐깁니다. 투숙객이 이용하려면 호텔 구역 안에 있어야 합니다.</t>
+        </is>
       </c>
     </row>
     <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15878,8 +15884,10 @@
       <c r="E18" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F18" s="2" t="s">
-        <v>76</v>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">투숙객끼리 겨루며, 카지노는 매 판에 모인 판돈에서 수수료를 가져갑니다. 위험이 적고 꾸준한 카지노 수입원입니다.\n\n의자가 필요합니다. 플레이어는 앉아서 게임을 하므로, 테이블 바로 옆에 플레이어마다 의자나 걸상을 하나씩 놓으세요. 최대 4명까지 이용할 수 있으며, 딜러는 필요 없습니다. 호텔 투숙객은 설정된 판돈을 자신의 예산에서 지불하고, 정착민은 재미로 즐깁니다. 투숙객이 이용하려면 호텔 구역 안에 있어야 합니다.</t>
+        </is>
       </c>
     </row>
     <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15912,8 +15920,10 @@
       <c r="E20" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="F20" s="2" t="s">
-        <v>84</v>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">주사위를 굴리며 소리쳐 보세요. 카지노에 돌아가는 이익이 적은 편인, 시끌벅적하게 함께 즐기는 게임입니다.\n\n의자가 필요합니다. 플레이어는 앉아서 게임을 하므로, 테이블 바로 옆에 플레이어마다 의자나 걸상을 하나씩 놓으세요. 최대 4명까지 이용할 수 있으며, 딜러는 필요 없습니다. 호텔 투숙객은 설정된 판돈을 자신의 예산에서 지불하고, 정착민은 재미로 즐깁니다. 투숙객이 이용하려면 호텔 구역 안에 있어야 합니다.</t>
+        </is>
       </c>
     </row>
     <row r="21" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15963,8 +15973,10 @@
       <c r="E23" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="F23" s="2" t="s">
-        <v>96</v>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">변방계 최고의 트럼보와 머팔로, 그리고 일직선으로 달릴 수 있는 온갖 동물들의 경주를 먼 경주장에서 중계하는 대형 화면입니다. 경주는 30분마다 열립니다. 호텔 투숙객은 설정된 판돈으로 참가 동물에게 돈을 걸고, 맞히면 판돈에 배당률을 곱한 금액을 받습니다. 당첨금 설정에 따라 카지노의 몫이 달라집니다. 좌석이 필요합니다. 투숙객은 앉아서 관람하므로, 화면 앞에 의자나 소파를 놓으세요. 최대 6명이 관람할 수 있습니다. 정착민은 경주 자체를 즐깁니다.\n\n경주 탭에서 다음 경주의 참가 동물과 배당률, 최근 결과를 볼 수 있습니다. 전력이 필요하며, 투숙객이 이용하려면 호텔 구역 안에 있어야 합니다.</t>
+        </is>
       </c>
     </row>
     <row r="24" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16320,8 +16332,10 @@
       <c r="E44" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="F44" s="2" t="s">
-        <v>181</v>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">좌석이 필요합니다. 투숙객은 앉아서만 관람하므로, 무대 앞 2~8칸 거리에 의자나 소파를 놓으세요. 화살표가 무대의 방향을 나타내며, 설치하거나 선택할 때 관람 구역이 표시됩니다.\n\n공연자를 위한 단상입니다. 호텔 탭의 공연자 페이지에서 지정한 정착민이 이곳에서 음악, 코미디, 마술 공연을 합니다. 공연의 수준은 예술, 사교, 연구 기술로 평가됩니다. 투숙객은 무대 앞 좌석에서 공연을 즐기며 자신의 예산에서 팁을 지불합니다. 실력 있는 공연자가 더 좋은 방에서 공연할수록 공연의 수준이 높아집니다. 정착민은 무료로 관람할 수 있습니다.\n\n정신력 증폭이 있는 마술사는 진짜 마술을 선보입니다. 공연 수준이 높아지고 잊지 못할 추억을 남기지만, 공연마다 초집중을 소모하고 신경열이 쌓입니다.\n\n호텔 구역 안에 있어야 합니다. 입장료를 받으려면 주변에 입장료 표지판을 놓으세요.</t>
+        </is>
       </c>
     </row>
     <row r="45" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18473,8 +18487,10 @@
       <c r="E162" s="2" t="s">
         <v>643</v>
       </c>
-      <c r="F162" s="2" t="s">
-        <v>644</v>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{PAWN_nameDef}(은)는 돈을 받고 함께 시간을 보내 주고 {PAWN_possessive} 몸을 파는 일을 거리끼지 않습니다. {PAWN_objective}에게는 그저 직업일 뿐이며, {PAWN_pronoun}(은)는 이 일을 전혀 싫어하지 않습니다.</t>
+        </is>
       </c>
     </row>
     <row r="163" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19734,8 +19750,10 @@
       <c r="E233" s="2" t="s">
         <v>920</v>
       </c>
-      <c r="F233" s="2" t="s">
-        <v>921</v>
+      <c r="F233" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">하루당 유흥 당일 방문 횟수: {0}</t>
+        </is>
       </c>
     </row>
     <row r="234" customFormat="false" ht="120.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19853,8 +19871,10 @@
       <c r="E240" s="2" t="s">
         <v>948</v>
       </c>
-      <c r="F240" s="2" t="s">
-        <v>949</v>
+      <c r="F240" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">커플들이 호텔에서 결혼식을 올리려고 연락합니다. 손님은 6~12명이며 2박 동안 머뭅니다. 호텔이 4성급(평판 80)이며 식당이 있어야 제안을 받습니다.\n\n첫날 저녁에 예식을 치를 수 있도록 호텔 구역 안에 결혼식 장소이 필요하며, 커플을 위한 디럭스 또는 스위트 객실의 2인용 침대가 필요합니다. 예식이 열리고, 모든 손님이 호텔 식당에서 식사하며, 숙박을 즐겼다면(만족도 60% 이상) 성공합니다. 은 보너스와 평판, 우호도를 얻습니다. 실패하면 평판이 조금 떨어지지만 예약금은 돌려주지 않아도 됩니다.\n\n0으로 설정하면 비활성화합니다.</t>
+        </is>
       </c>
     </row>
     <row r="241" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20006,8 +20026,10 @@
       <c r="E249" s="2" t="s">
         <v>984</v>
       </c>
-      <c r="F249" s="2" t="s">
-        <v>985</v>
+      <c r="F249" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">영연방식 명칭 사용 (스태그 파티, 헨 파티)</t>
+        </is>
       </c>
     </row>
     <row r="250" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20023,8 +20045,10 @@
       <c r="E250" s="2" t="s">
         <v>988</v>
       </c>
-      <c r="F250" s="2" t="s">
-        <v>989</v>
+      <c r="F250" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">켜짐: 예비 신랑의 파티는 스태그 파티(stag do), 예비 신부의 파티는 헨 파티(hen do)라고 부릅니다.\n\n꺼짐: 총각 파티(bachelor party)와 처녀 파티(bachelorette party)라고 부릅니다.\n\n단일 성별 파티를 끈 경우, 남녀가 함께하는 파티는 항상 결혼 전 파티라고 부릅니다.</t>
+        </is>
       </c>
     </row>
     <row r="251" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21094,8 +21118,10 @@
       <c r="E313" s="2" t="s">
         <v>1235</v>
       </c>
-      <c r="F313" s="2" t="s">
-        <v>1236</v>
+      <c r="F313" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{0} 소속 손님들이 예약을 취소했습니다. 이곳이 너무 위험한 상태였습니다.</t>
+        </is>
       </c>
     </row>
     <row r="314" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21196,8 +21222,10 @@
       <c r="E319" s="2" t="s">
         <v>1257</v>
       </c>
-      <c r="F319" s="2" t="s">
-        <v>1258</v>
+      <c r="F319" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">호텔 투숙객이 이곳에서 자판기처럼 호텔의 영양죽 가격으로 영양죽을 구매할 수 있습니다. 정착민은 계속 무료로 이용합니다. 호텔 구역 안에서만 작동합니다.</t>
+        </is>
       </c>
     </row>
     <row r="320" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23151,8 +23179,10 @@
       <c r="E434" s="2" t="s">
         <v>1714</v>
       </c>
-      <c r="F434" s="2" t="s">
-        <v>1715</v>
+      <c r="F434" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{1} 소속 커플이 호텔에서 결혼식을 올리고 싶어 합니다. 손님 {0}명이 {2}에 도착하여 2박 동안 머뭅니다. 예식은 첫날 저녁 약 {8}:00에 호텔 구역 안의 결혼식 장소에서 열립니다.\n\n성공 조건: 예식이 열리고, 모든 손님이 호텔 식당에서 한 번 이상 식사하며, 커플이 신혼 객실로 디럭스 또는 스위트 등급의 2인용 침대를 받고, 손님들이 숙박을 즐겨야 합니다(만족도 {7} 이상).\n\n수락하면 지금 예약금 {3}을 받습니다. 성공하면 보너스 {4}을 받고 평판이 {5} 상승하며, 해당 세력의 평가도 좋아집니다. 실패하면 평판이 {6} 감소합니다. 예약금은 돌려주지 않아도 됩니다.</t>
+        </is>
       </c>
     </row>
     <row r="435" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23168,8 +23198,10 @@
       <c r="E435" s="2" t="s">
         <v>1718</v>
       </c>
-      <c r="F435" s="2" t="s">
-        <v>1719</v>
+      <c r="F435" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">아직 호텔 구역 안에 결혼식 장소이 없습니다. 예식 전에 기타 메뉴에서 설치하세요.</t>
+        </is>
       </c>
     </row>
     <row r="436" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23236,8 +23268,10 @@
       <c r="E439" s="2" t="s">
         <v>1734</v>
       </c>
-      <c r="F439" s="2" t="s">
-        <v>1735</v>
+      <c r="F439" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{0}의 결혼식이 시작됩니다. 손님들이 결혼식 장소에 모이고 있습니다.</t>
+        </is>
       </c>
     </row>
     <row r="440" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23270,8 +23304,10 @@
       <c r="E441" s="2" t="s">
         <v>1742</v>
       </c>
-      <c r="F441" s="2" t="s">
-        <v>1743</v>
+      <c r="F441" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{0}의 결혼식을 시작할 수 없습니다. 호텔 구역 안에 결혼식 장소이 없습니다. 설치하면 예식이 시작됩니다.</t>
+        </is>
       </c>
     </row>
     <row r="442" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23321,8 +23357,10 @@
       <c r="E444" s="2" t="s">
         <v>1754</v>
       </c>
-      <c r="F444" s="2" t="s">
-        <v>1755</v>
+      <c r="F444" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">호텔 구역 안에 결혼식 장소이 마련되지 않았습니다.</t>
+        </is>
       </c>
     </row>
     <row r="445" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23338,8 +23376,10 @@
       <c r="E445" s="2" t="s">
         <v>1758</v>
       </c>
-      <c r="F445" s="2" t="s">
-        <v>1759</v>
+      <c r="F445" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">커플이 결혼식 장소에 도착하지 못했습니다.</t>
+        </is>
       </c>
     </row>
     <row r="446" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23508,8 +23548,10 @@
       <c r="E455" s="2" t="s">
         <v>1796</v>
       </c>
-      <c r="F455" s="2" t="s">
-        <v>1797</v>
+      <c r="F455" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">결혼식 장소 대기 중</t>
+        </is>
       </c>
     </row>
     <row r="456" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23644,8 +23686,10 @@
       <c r="E463" s="2" t="s">
         <v>1828</v>
       </c>
-      <c r="F463" s="2" t="s">
-        <v>1829</v>
+      <c r="F463" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{1} 등급 침대 {0}개를 {2} 등급으로 변경 가능</t>
+        </is>
       </c>
     </row>
     <row r="464" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23695,8 +23739,10 @@
       <c r="E466" s="2" t="s">
         <v>1840</v>
       </c>
-      <c r="F466" s="2" t="s">
-        <v>1841</v>
+      <c r="F466" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">침대 옆의 협탁이나 옷장, 또는 방 안의 장식이나 오락 시설</t>
+        </is>
       </c>
     </row>
     <row r="467" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23712,8 +23758,10 @@
       <c r="E467" s="2" t="s">
         <v>1844</v>
       </c>
-      <c r="F467" s="2" t="s">
-        <v>1845</v>
+      <c r="F467" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">침대 옆의 협탁이나 옷장</t>
+        </is>
       </c>
     </row>
     <row r="468" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23729,8 +23777,10 @@
       <c r="E468" s="2" t="s">
         <v>1848</v>
       </c>
-      <c r="F468" s="2" t="s">
-        <v>1849</v>
+      <c r="F468" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">침대용 가구 하나 더 (협탁과 옷장 모두 필요)</t>
+        </is>
       </c>
     </row>
     <row r="469" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23797,8 +23847,10 @@
       <c r="E472" s="2" t="s">
         <v>1864</v>
       </c>
-      <c r="F472" s="2" t="s">
-        <v>1865</v>
+      <c r="F472" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">각 등급의 필요 조건입니다. 별도로 방 인상 수치도 필요합니다(스탠더드 25, 디럭스 50, 스위트 90).\n- 스탠더드: 침대 옆의 협탁이나 옷장, 또는 방 안의 장식이나 오락 시설(예술품, TV 등 오락 시설, 화분)\n- 디럭스: 침대용 가구와 장식 또는 오락 시설\n- 스위트: 협탁과 옷장, 장식 또는 오락 시설, 상급 이상의 침대, 단독 객실(침대 1개)\n\n가구와 침대의 품질은 손님이 생각하는 1박의 가치도 높여 줍니다.</t>
+        </is>
       </c>
     </row>
     <row r="473" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24137,8 +24189,10 @@
       <c r="E492" s="2" t="s">
         <v>1941</v>
       </c>
-      <c r="F492" s="2" t="s">
-        <v>1942</v>
+      <c r="F492" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자판기 숨기기</t>
+        </is>
       </c>
     </row>
     <row r="493" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24783,8 +24837,10 @@
       <c r="E530" s="2" t="s">
         <v>2093</v>
       </c>
-      <c r="F530" s="2" t="s">
-        <v>2094</v>
+      <c r="F530" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">식당이나 자판기가 없습니다. 손님은 음식을 가져오지 않아 굶게 됩니다. 호텔 구역 안에 기타 메뉴의 식당 표지판이나 자판기를 설치하세요.</t>
+        </is>
       </c>
     </row>
     <row r="531" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24800,8 +24856,10 @@
       <c r="E531" s="2" t="s">
         <v>2097</v>
       </c>
-      <c r="F531" s="2" t="s">
-        <v>2098</v>
+      <c r="F531" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">호텔 구역 안의 식당과 자판기 어디에도 음식 재고가 없습니다. 손님이 굶게 됩니다.</t>
+        </is>
       </c>
     </row>
     <row r="532" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27537,8 +27595,10 @@
       <c r="E692" s="2" t="s">
         <v>2732</v>
       </c>
-      <c r="F692" s="2" t="s">
-        <v>2733</v>
+      <c r="F692" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">모든 식당, 상점, 자판기</t>
+        </is>
       </c>
     </row>
     <row r="693" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27554,8 +27614,10 @@
       <c r="E693" s="2" t="s">
         <v>2736</v>
       </c>
-      <c r="F693" s="2" t="s">
-        <v>2737</v>
+      <c r="F693" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">끄면 이 패키지의 손님이 이용할 식당, 상점, 자판기를 직접 선택할 수 있습니다.</t>
+        </is>
       </c>
     </row>
     <row r="694" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27571,8 +27633,10 @@
       <c r="E694" s="2" t="s">
         <v>2740</v>
       </c>
-      <c r="F694" s="2" t="s">
-        <v>2741</v>
+      <c r="F694" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">아직 호텔 구역 안에 식당, 상점, 자판기가 없습니다.</t>
+        </is>
       </c>
     </row>
     <row r="695" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27707,8 +27771,10 @@
       <c r="E702" s="2" t="s">
         <v>2772</v>
       </c>
-      <c r="F702" s="2" t="s">
-        <v>2773</v>
+      <c r="F702" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">식당, 자판기, 영양죽 분배기에서 구매하는 음식에 적용하는 할인입니다. 포함된 식사는 계속 무료입니다.\n\n이곳의 일반적인 손님은 식비로 1박당 약 {0}을 쓰므로, 약 {1}을 절약합니다. 포함된 식사가 이미 충당하는 부분은 제외합니다. 이 절약액은 패키지 가치에 반영됩니다.</t>
+        </is>
       </c>
     </row>
     <row r="703" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27724,8 +27790,10 @@
       <c r="E703" s="2" t="s">
         <v>2776</v>
       </c>
-      <c r="F703" s="2" t="s">
-        <v>2777</v>
+      <c r="F703" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">상점과 식사 대신 쇼핑 목적으로 이용하는 자판기에 적용하는 할인입니다.\n\n이곳의 일반적인 손님은 쇼핑에 1박당 약 {0}을 쓰므로, 약 {1}을 절약합니다. 이 절약액은 패키지 가치에 반영됩니다.</t>
+        </is>
       </c>
     </row>
     <row r="704" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28863,8 +28931,10 @@
       <c r="E770" s="2" t="s">
         <v>3028</v>
       </c>
-      <c r="F770" s="2" t="s">
-        <v>3029</v>
+      <c r="F770" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">은으로 결제합니다. 언제나 사용 가능하며 수수료가 없습니다. 원시, 중세, 산업 기술 수준의 손님 대부분이 사용합니다. 우주 기술 수준의 손님은 구식이라고 여깁니다.</t>
+        </is>
       </c>
     </row>
     <row r="771" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28897,8 +28967,10 @@
       <c r="E772" s="2" t="s">
         <v>3036</v>
       </c>
-      <c r="F772" s="2" t="s">
-        <v>3037</v>
+      <c r="F772" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">안목 있는 여행자를 위한 InterRim Bank입니다. 우주 기술 수준의 손님이 선호합니다. 미래 기술 수준의 손님은 이 방식으로만 결제하며, 이를 받지 않는 호텔에는 오지 않습니다. 초기 가입비와 수수료가 더 높습니다.</t>
+        </is>
       </c>
     </row>
     <row r="773" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29237,8 +29309,10 @@
       <c r="E792" s="2" t="s">
         <v>3116</v>
       </c>
-      <c r="F792" s="2" t="s">
-        <v>3117</v>
+      <c r="F792" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">손님이 속한 세력의 기술 수준에 따라 달라집니다.\n- 원시 및 중세: 현금만 사용합니다.\n- 산업: 현금과 RimCard 모두 괜찮습니다.\n- 우주: InterRim Bank, RimCard, 현금 순으로 사용하며 현금을 싫어합니다.\n- 미래 이상: InterRim Bank만 사용합니다. 받지 않으면 해당 세력은 손님을 보내지 않습니다.</t>
+        </is>
       </c>
     </row>
     <row r="793" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29560,8 +29634,10 @@
       <c r="E811" s="2" t="s">
         <v>3184</v>
       </c>
-      <c r="F811" s="2" t="s">
-        <v>3185</v>
+      <c r="F811" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">다른 행성에서 온 부유한 손님입니다. 우주 기술 수준이며, InterRim Bank를 받으면 미래 기술 수준의 손님도 옵니다. 우주선에서 전송되어 내려오고, 떠날 때 다시 전송되어 올라갑니다. 호텔 구역 안에 전송 도착 지점이 필요하며, 일반 예산의 세 배를 가져옵니다.</t>
+        </is>
       </c>
     </row>
     <row r="812" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31362,8 +31438,10 @@
       <c r="E917" s="2" t="s">
         <v>3600</v>
       </c>
-      <c r="F917" s="2" t="s">
-        <v>3601</v>
+      <c r="F917" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">아직 카지노 게임이 없습니다. 호텔 구역 안에 슬롯머신, 동전 밀어내기 기계, 카지노 테이블, 경주 베팅 전광판을 설치하세요 (오락 탭).</t>
+        </is>
       </c>
     </row>
     <row r="918" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31719,8 +31797,10 @@
       <c r="E938" s="2" t="s">
         <v>3682</v>
       </c>
-      <c r="F938" s="2" t="s">
-        <v>3683</v>
+      <c r="F938" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">하루당 카지노 당일 방문 횟수: {0}</t>
+        </is>
       </c>
     </row>
     <row r="939" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32178,8 +32258,10 @@
       <c r="E965" s="2" t="s">
         <v>3790</v>
       </c>
-      <c r="F965" s="2" t="s">
-        <v>3791</v>
+      <c r="F965" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">카지노 결과 알림 표시</t>
+        </is>
       </c>
     </row>
     <row r="966" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32348,8 +32430,10 @@
       <c r="E975" s="2" t="s">
         <v>3829</v>
       </c>
-      <c r="F975" s="2" t="s">
-        <v>3830</v>
+      <c r="F975" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">공연자는 호텔 구역의 공연 무대에서 음악(예술), 코미디(사교), 마술(연구) 공연을 합니다. 음악을 맡은 연주자는 무대보다 가까우면 호텔 구역의 악기를 연주할 수도 있습니다. 하프, 하프시코드, 피아노, 북, 모드로 추가한 악기를 사용할 수 있습니다. 손님은 앉아서만 듣습니다. 악기와 같은 방 안의 9칸 이내에 의자를 놓으세요. 악기를 선택하면 범위가 보입니다. 접객을 맡은 담당자는 사교 기술을 사용하며 무대가 필요 없습니다. 호텔을 돌아다니며 한가하거나 오락 활동 중인 손님과 대화합니다. 새로 도착한 손님을 먼저 환영한 뒤, 숙박 만족도가 가장 낮은 손님을 위로합니다. 접객은 무료이며, 좋은 담당자는 손님에게 행복한 기억을 남깁니다. 무대 공연도 손님이 앉아서 관람하므로, 무대 앞 2~8칸 거리에 의자나 소파가 필요합니다. 무대를 선택하면 범위가 보입니다. 손님은 즐거운 시간을 보내고 좋은 공연을 기억하며, 자신의 예산에서 팁을 줍니다. 기술이 높고 방이 더 인상적일수록 공연 수준이 높아집니다. 정착민은 무료로 관람할 수 있습니다.\n\n각 공연자에게는 근무 방식이 있습니다.\n- 공연 시간: 시간표와 관계없이 막대에 지정한 시간에 공연합니다.\n- 전일제: 손님이 있는 동안 시간표의 작업 및 자유행동 시간에 공연합니다.\n- 시간제: 오락 시간에 공연하며, 자유행동 시간에는 다른 할 일이 없을 때만 공연합니다.\n\n입장료를 받으려면 무대 주변에 입장료 표지판을 놓으세요.</t>
+        </is>
       </c>
     </row>
     <row r="976" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32552,8 +32636,10 @@
       <c r="E987" s="2" t="s">
         <v>3875</v>
       </c>
-      <c r="F987" s="2" t="s">
-        <v>3876</v>
+      <c r="F987" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전일제: 손님이 있는 동안 작업 및 자유행동 시간에 공연합니다.</t>
+        </is>
       </c>
     </row>
     <row r="988" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32569,8 +32655,10 @@
       <c r="E988" s="2" t="s">
         <v>3879</v>
       </c>
-      <c r="F988" s="2" t="s">
-        <v>3880</v>
+      <c r="F988" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">시간제: 손님이 있는 동안 오락 시간에 공연하며, 자유행동 시간에는 다른 할 일이 없을 때만 공연합니다.</t>
+        </is>
       </c>
     </row>
     <row r="989" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33396,8 +33484,10 @@
       <c r="E1034" s="2" t="s">
         <v>4058</v>
       </c>
-      <c r="F1034" s="2" t="s">
-        <v>4059</v>
+      <c r="F1034" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{0}(은)는 성매매를 원하지 않습니다.\n\n{1}\n\n{PAWN_objective}에게 강요하면:\n- {PAWN_pronoun}(은)는 {PAWN_pronoun} 자신이 강요받는 동안 계속 비참해합니다.\n- {PAWN_pronoun}(은)는 이를 방치한 다른 모든 정착민을 원망합니다.\n- 모든 접대는 비동의 행위로 집계됩니다.\n\n그래도 {0}에게 강요하시겠습니까?</t>
+        </is>
       </c>
     </row>
     <row r="1035" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33436,8 +33526,10 @@
       <c r="E1036" s="2" t="s">
         <v>4066</v>
       </c>
-      <c r="F1036" s="2" t="s">
-        <v>4067</v>
+      <c r="F1036" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">이 정착민이 호텔 손님을 접대하도록 합니다. 손님은 시간표가 작업 또는 자유행동인 근무 중의 접대부를 예약하며, 접대마다 비용을 지불합니다.\n\n이 일을 원하는 정착민만 맡아야 합니다.</t>
+        </is>
       </c>
     </row>
     <row r="1037" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35396,8 +35488,12 @@
       <c r="E1134" s="2" t="s">
         <v>4439</v>
       </c>
-      <c r="F1134" s="2" t="s">
-        <v>4440</v>
+      <c r="F1134" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">시간제 접대부는 평소의 작업을 유지합니다. 시간표의 오락 또는 자유행동 시간에만 접대하며, 일하지 않고 한가할 때만 예약을 받습니다. 무용수는 오락 시간에 춤추며, 자유행동 시간에는 할 일이 없을 때만 춤춥니다.
+전일제 접대부는 작업 또는 자유행동 시간에 근무하며, 접대와 춤이 다른 작업보다 우선합니다.
+가격과 윤리 점수는 두 방식 모두 동일하게 적용합니다.</t>
+        </is>
       </c>
     </row>
     <row r="1135" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35496,8 +35592,10 @@
       <c r="E1139" s="2" t="s">
         <v>4457</v>
       </c>
-      <c r="F1139" s="2" t="s">
-        <v>4458</v>
+      <c r="F1139" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">변방계를 걱정하는 시민들</t>
+        </is>
       </c>
     </row>
     <row r="1140" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -36376,8 +36474,10 @@
       <c r="E1183" s="2" t="s">
         <v>4630</v>
       </c>
-      <c r="F1183" s="2" t="s">
-        <v>4631</v>
+      <c r="F1183" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">성적 접대 요금을 현금으로만 받습니다. {0}의 압박 활동을 끝내는 주된 방법이며, 새로운 압박도 막습니다.\n\n손님은 다른 곳에서와 같은 방식으로 결제합니다. 산업 기술 수준의 손님은 현금을 기꺼이 사용하고, 우주 기술 수준의 손님은 마지못해 사용하며 무드가 나빠집니다. 미래 기술 수준의 손님은 현금을 갖고 다니지 않아 접대를 예약할 수 없습니다.</t>
+        </is>
       </c>
     </row>
     <row r="1184" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -37336,8 +37436,10 @@
       <c r="E1231" s="2" t="s">
         <v>4816</v>
       </c>
-      <c r="F1231" s="2" t="s">
-        <v>4817</v>
+      <c r="F1231" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">근무 시간(시간표의 작업 또는 자유행동)에 손님 예약이 없으면 호텔 구역의 스트립 폴에서 춤을 춥니다. 관람하는 손님은 자신의 예산에서 팁을 주며, 마음에 드는 무용수를 예약하는 경우가 많습니다.</t>
+        </is>
       </c>
     </row>
     <row r="1232" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -37576,8 +37678,10 @@
       <c r="E1243" s="2" t="s">
         <v>4864</v>
       </c>
-      <c r="F1243" s="2" t="s">
-        <v>4865</v>
+      <c r="F1243" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">일행은 {0} 후 객실을 예약해 하룻밤 머물지 결정합니다. 현재 확률은 {1}이며, 즐거운 시간을 보내고 모두가 한 번 이상 접대를 받으면 높아집니다.</t>
+        </is>
       </c>
     </row>
     <row r="1244" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -37636,8 +37740,10 @@
       <c r="E1246" s="2" t="s">
         <v>4876</v>
       </c>
-      <c r="F1246" s="2" t="s">
-        <v>4869</v>
+      <c r="F1246" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">스태그 파티</t>
+        </is>
       </c>
     </row>
     <row r="1247" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -37656,8 +37762,10 @@
       <c r="E1247" s="2" t="s">
         <v>4879</v>
       </c>
-      <c r="F1247" s="2" t="s">
-        <v>4873</v>
+      <c r="F1247" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">헨 파티</t>
+        </is>
       </c>
     </row>
     <row r="1248" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -38376,8 +38484,10 @@
       <c r="E1283" s="2" t="s">
         <v>5018</v>
       </c>
-      <c r="F1283" s="2" t="s">
-        <v>5019</v>
+      <c r="F1283" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">호텔 구역에 변기이 없어 손님이 야외에서 볼일을 봅니다.</t>
+        </is>
       </c>
     </row>
     <row r="1284" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -38436,8 +38546,10 @@
       <c r="E1286" s="2" t="s">
         <v>5030</v>
       </c>
-      <c r="F1286" s="2" t="s">
-        <v>5031</v>
+      <c r="F1286" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">이 방 안에 있거나, 유일한 문이 이 방으로 통하는 전용 욕실에 있는 변기, 샤워기, 욕조, 세면대를 이 방의 투숙객용 침대에 연결합니다. 그러면 이 객실의 투숙객만 이용합니다.\n\n호텔은 매시간 자동으로 연결하며, 이 버튼은 즉시 연결합니다. 이미 정착민의 침대에 연결된 시설은 그대로 둡니다.</t>
+        </is>
       </c>
     </row>
     <row r="1287" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -38496,8 +38608,10 @@
       <c r="E1289" s="2" t="s">
         <v>5042</v>
       </c>
-      <c r="F1289" s="2" t="s">
-        <v>5043</v>
+      <c r="F1289" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">이 방이나 연결된 전용 욕실에 변기, 샤워기, 욕조, 세면대가 없습니다.</t>
+        </is>
       </c>
     </row>
     <row r="1290" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -38516,8 +38630,10 @@
       <c r="E1290" s="2" t="s">
         <v>5046</v>
       </c>
-      <c r="F1290" s="2" t="s">
-        <v>5047</v>
+      <c r="F1290" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전용 욕실 (객실 안이나 연결된 전용 욕실에 변기와 샤워기 또는 욕조 필요)</t>
+        </is>
       </c>
     </row>
     <row r="1291" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -38536,8 +38652,10 @@
       <c r="E1291" s="2" t="s">
         <v>5050</v>
       </c>
-      <c r="F1291" s="2" t="s">
-        <v>5051</v>
+      <c r="F1291" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dubs Bad Hygiene 사용 시: 디럭스와 스위트는 전용 욕실도 필요합니다. 변기과 샤워기 또는 욕조가 객실 안에 있거나, 유일한 문이 해당 객실로 통하는 전용 욕실에 있어야 합니다.</t>
+        </is>
       </c>
     </row>
     <row r="1292" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>